<commit_message>
Date and Time standardization
</commit_message>
<xml_diff>
--- a/ticketing-system/dataset/tickets-v1.xlsx
+++ b/ticketing-system/dataset/tickets-v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e29a6debf5eaf8e/Documents/GitHub/northstar-health-operations/ticketing-system/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{7DEB1219-D846-4A40-83BF-C89E2A7D2CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDE587E1-9138-4956-8ECA-2930C86C4386}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{7DEB1219-D846-4A40-83BF-C89E2A7D2CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D99413E3-1132-4950-BD68-7523471CB13D}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="16515" windowHeight="16380" xr2:uid="{2C631232-D7C3-4194-A702-1BFDC8C8A37B}"/>
+    <workbookView xWindow="4650" yWindow="1635" windowWidth="16515" windowHeight="16380" xr2:uid="{2C631232-D7C3-4194-A702-1BFDC8C8A37B}"/>
   </bookViews>
   <sheets>
     <sheet name="tickets-v1" sheetId="1" r:id="rId1"/>
@@ -293,9 +293,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:m"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:m"/>
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -774,10 +775,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1160,8 +1162,8 @@
   <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
   </cols>
@@ -1173,7 +1175,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -1235,7 +1237,7 @@
       <c r="B2" s="1">
         <v>46162</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="3">
         <v>46162.35</v>
       </c>
       <c r="D2" s="2">
@@ -1297,7 +1299,7 @@
       <c r="B3" s="1">
         <v>46162</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="3">
         <v>46162.402777777781</v>
       </c>
       <c r="D3" s="2">
@@ -1359,7 +1361,7 @@
       <c r="B4" s="1">
         <v>46162</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="3">
         <v>46162.436805555553</v>
       </c>
       <c r="D4" s="2">
@@ -1421,7 +1423,7 @@
       <c r="B5" s="1">
         <v>46162</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="3">
         <v>46162.496527777781</v>
       </c>
       <c r="F5" t="s">
@@ -1468,7 +1470,7 @@
       <c r="B6" s="1">
         <v>46162</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="3">
         <v>46162.577777777777</v>
       </c>
       <c r="D6" s="2">
@@ -1530,7 +1532,7 @@
       <c r="B7" s="1">
         <v>46162</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="3">
         <v>46162.600694444445</v>
       </c>
       <c r="D7" s="2">
@@ -1592,7 +1594,7 @@
       <c r="B8" s="1">
         <v>46162</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="3">
         <v>46162.686111111114</v>
       </c>
       <c r="F8" t="s">
@@ -1639,7 +1641,7 @@
       <c r="B9" s="1">
         <v>46162</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="3">
         <v>46162.695138888892</v>
       </c>
       <c r="D9" s="2">
@@ -1701,7 +1703,7 @@
       <c r="B10" s="1">
         <v>46162</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="3">
         <v>46162.756944444445</v>
       </c>
       <c r="D10" s="2">
@@ -1763,7 +1765,7 @@
       <c r="B11" s="1">
         <v>46162</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="3">
         <v>46162.78125</v>
       </c>
       <c r="D11" s="2">
@@ -1825,7 +1827,7 @@
       <c r="B12" s="1">
         <v>46163</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="3">
         <v>46163.320833333331</v>
       </c>
       <c r="D12" s="2">
@@ -1887,7 +1889,7 @@
       <c r="B13" s="1">
         <v>46163</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="3">
         <v>46163.371527777781</v>
       </c>
       <c r="F13" t="s">
@@ -1934,7 +1936,7 @@
       <c r="B14" s="1">
         <v>46163</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="3">
         <v>46163.429166666669</v>
       </c>
       <c r="D14" s="2">
@@ -1996,7 +1998,7 @@
       <c r="B15" s="1">
         <v>46163</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="3">
         <v>46163.48541666667</v>
       </c>
       <c r="D15" s="2">
@@ -2058,7 +2060,7 @@
       <c r="B16" s="1">
         <v>46163</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="3">
         <v>46163.501388888886</v>
       </c>
       <c r="F16" t="s">
@@ -2100,5 +2102,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update lost time on tickets-v1
</commit_message>
<xml_diff>
--- a/ticketing-system/dataset/tickets-v1.xlsx
+++ b/ticketing-system/dataset/tickets-v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e29a6debf5eaf8e/Documents/GitHub/northstar-health-operations/ticketing-system/dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{7DEB1219-D846-4A40-83BF-C89E2A7D2CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D99413E3-1132-4950-BD68-7523471CB13D}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{7DEB1219-D846-4A40-83BF-C89E2A7D2CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C365ABD-800B-418D-B61E-1C3AD2752879}"/>
   <bookViews>
-    <workbookView xWindow="4650" yWindow="1635" windowWidth="16515" windowHeight="16380" xr2:uid="{2C631232-D7C3-4194-A702-1BFDC8C8A37B}"/>
+    <workbookView xWindow="3405" yWindow="1980" windowWidth="16515" windowHeight="16380" xr2:uid="{2C631232-D7C3-4194-A702-1BFDC8C8A37B}"/>
   </bookViews>
   <sheets>
     <sheet name="tickets-v1" sheetId="1" r:id="rId1"/>
@@ -293,10 +293,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  <numFmts count="2">
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:m"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -777,9 +776,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1162,26 +1161,26 @@
   <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1234,16 +1233,16 @@
       <c r="A2" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C2" s="3">
+      <c r="B2" s="3">
+        <v>46162.341666666667</v>
+      </c>
+      <c r="C2" s="2">
         <v>46162.35</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>46162.447916666664</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>46162.459722222222</v>
       </c>
       <c r="F2" t="s">
@@ -1296,16 +1295,16 @@
       <c r="A3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="B3" s="3">
+        <v>46162.377083333333</v>
+      </c>
+      <c r="C3" s="2">
         <v>46162.402777777781</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>46163.59375</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>46163.612500000003</v>
       </c>
       <c r="F3" t="s">
@@ -1358,16 +1357,16 @@
       <c r="A4" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C4" s="3">
+      <c r="B4" s="3">
+        <v>46162.424305555556</v>
+      </c>
+      <c r="C4" s="2">
         <v>46162.436805555553</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>46162.574999999997</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>46162.585416666669</v>
       </c>
       <c r="F4" t="s">
@@ -1420,10 +1419,10 @@
       <c r="A5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="B5" s="3">
+        <v>46162.476388888892</v>
+      </c>
+      <c r="C5" s="2">
         <v>46162.496527777781</v>
       </c>
       <c r="F5" t="s">
@@ -1467,16 +1466,16 @@
       <c r="A6" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C6" s="3">
+      <c r="B6" s="3">
+        <v>46162.554166666669</v>
+      </c>
+      <c r="C6" s="2">
         <v>46162.577777777777</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>46163.384722222225</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>46163.402777777781</v>
       </c>
       <c r="F6" t="s">
@@ -1529,16 +1528,16 @@
       <c r="A7" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C7" s="3">
+      <c r="B7" s="3">
+        <v>46162.584722222222</v>
+      </c>
+      <c r="C7" s="2">
         <v>46162.600694444445</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>46162.679166666669</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>46162.694444444445</v>
       </c>
       <c r="F7" t="s">
@@ -1591,10 +1590,10 @@
       <c r="A8" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C8" s="3">
+      <c r="B8" s="3">
+        <v>46162.655555555553</v>
+      </c>
+      <c r="C8" s="2">
         <v>46162.686111111114</v>
       </c>
       <c r="F8" t="s">
@@ -1638,16 +1637,16 @@
       <c r="A9" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C9" s="3">
+      <c r="B9" s="3">
+        <v>46162.677083333336</v>
+      </c>
+      <c r="C9" s="2">
         <v>46162.695138888892</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>46162.751388888886</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>46162.762499999997</v>
       </c>
       <c r="F9" t="s">
@@ -1700,16 +1699,16 @@
       <c r="A10" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C10" s="3">
+      <c r="B10" s="3">
+        <v>46162.730555555558</v>
+      </c>
+      <c r="C10" s="2">
         <v>46162.756944444445</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>46163.362500000003</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>46163.382638888892</v>
       </c>
       <c r="F10" t="s">
@@ -1762,16 +1761,16 @@
       <c r="A11" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="1">
-        <v>46162</v>
-      </c>
-      <c r="C11" s="3">
+      <c r="B11" s="3">
+        <v>46162.75277777778</v>
+      </c>
+      <c r="C11" s="2">
         <v>46162.78125</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>46164.470833333333</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46164.490972222222</v>
       </c>
       <c r="F11" t="s">
@@ -1824,16 +1823,16 @@
       <c r="A12" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="1">
-        <v>46163</v>
-      </c>
-      <c r="C12" s="3">
+      <c r="B12" s="3">
+        <v>46163.304166666669</v>
+      </c>
+      <c r="C12" s="2">
         <v>46163.320833333331</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>46163.380555555559</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46163.393055555556</v>
       </c>
       <c r="F12" t="s">
@@ -1886,10 +1885,10 @@
       <c r="A13" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="1">
-        <v>46163</v>
-      </c>
-      <c r="C13" s="3">
+      <c r="B13" s="3">
+        <v>46163.34097222222</v>
+      </c>
+      <c r="C13" s="2">
         <v>46163.371527777781</v>
       </c>
       <c r="F13" t="s">
@@ -1933,16 +1932,16 @@
       <c r="A14" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="1">
-        <v>46163</v>
-      </c>
-      <c r="C14" s="3">
+      <c r="B14" s="3">
+        <v>46163.405555555553</v>
+      </c>
+      <c r="C14" s="2">
         <v>46163.429166666669</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>46163.54791666667</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46163.56527777778</v>
       </c>
       <c r="F14" t="s">
@@ -1995,16 +1994,16 @@
       <c r="A15" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="1">
-        <v>46163</v>
-      </c>
-      <c r="C15" s="3">
+      <c r="B15" s="3">
+        <v>46163.452777777777</v>
+      </c>
+      <c r="C15" s="2">
         <v>46163.48541666667</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>46164.654166666667</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46164.673611111109</v>
       </c>
       <c r="F15" t="s">
@@ -2057,10 +2056,10 @@
       <c r="A16" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="1">
-        <v>46163</v>
-      </c>
-      <c r="C16" s="3">
+      <c r="B16" s="3">
+        <v>46163.481249999997</v>
+      </c>
+      <c r="C16" s="2">
         <v>46163.501388888886</v>
       </c>
       <c r="F16" t="s">

</xml_diff>